<commit_message>
ingesta: snapshot 2026-07-16 18:35 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-16/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-16/CORDOBA_JUL26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC83B054-216D-4C77-BCDA-4E0D2A6E362F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448DCEAF-AC30-4CFF-8B38-FB472E8870E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
@@ -7393,7 +7393,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7866,7 +7866,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -8470,7 +8470,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9079,7 +9079,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9689,7 +9689,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -10002,7 +10002,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>-1</c:v>
@@ -19961,7 +19961,9 @@
       <c r="R3" s="25">
         <v>0</v>
       </c>
-      <c r="S3" s="25"/>
+      <c r="S3" s="25">
+        <v>0</v>
+      </c>
       <c r="T3" s="25"/>
       <c r="U3" s="25"/>
       <c r="V3" s="25"/>
@@ -20041,7 +20043,9 @@
       <c r="R4" s="25">
         <v>0</v>
       </c>
-      <c r="S4" s="25"/>
+      <c r="S4" s="25">
+        <v>0</v>
+      </c>
       <c r="T4" s="25"/>
       <c r="U4" s="25"/>
       <c r="V4" s="25"/>
@@ -20121,7 +20125,9 @@
       <c r="R5" s="25">
         <v>0</v>
       </c>
-      <c r="S5" s="25"/>
+      <c r="S5" s="25">
+        <v>0</v>
+      </c>
       <c r="T5" s="25"/>
       <c r="U5" s="25"/>
       <c r="V5" s="25"/>
@@ -20201,7 +20207,9 @@
       <c r="R6" s="25">
         <v>0</v>
       </c>
-      <c r="S6" s="25"/>
+      <c r="S6" s="25">
+        <v>0</v>
+      </c>
       <c r="T6" s="25"/>
       <c r="U6" s="25"/>
       <c r="V6" s="25"/>
@@ -20385,7 +20393,9 @@
       <c r="R9" s="25">
         <v>0</v>
       </c>
-      <c r="S9" s="25"/>
+      <c r="S9" s="25">
+        <v>0</v>
+      </c>
       <c r="T9" s="25"/>
       <c r="U9" s="25"/>
       <c r="V9" s="25"/>
@@ -20543,7 +20553,9 @@
       <c r="R11" s="25">
         <v>0</v>
       </c>
-      <c r="S11" s="25"/>
+      <c r="S11" s="25">
+        <v>0</v>
+      </c>
       <c r="T11" s="25"/>
       <c r="U11" s="25"/>
       <c r="V11" s="25"/>
@@ -20621,7 +20633,9 @@
       <c r="R12" s="25">
         <v>0</v>
       </c>
-      <c r="S12" s="25"/>
+      <c r="S12" s="25">
+        <v>0</v>
+      </c>
       <c r="T12" s="25"/>
       <c r="U12" s="25"/>
       <c r="V12" s="25"/>
@@ -20701,7 +20715,9 @@
       <c r="R13" s="25">
         <v>0</v>
       </c>
-      <c r="S13" s="25"/>
+      <c r="S13" s="25">
+        <v>0</v>
+      </c>
       <c r="T13" s="25"/>
       <c r="U13" s="25"/>
       <c r="V13" s="25"/>
@@ -20779,7 +20795,9 @@
       <c r="R14" s="25">
         <v>0</v>
       </c>
-      <c r="S14" s="25"/>
+      <c r="S14" s="25">
+        <v>0</v>
+      </c>
       <c r="T14" s="25"/>
       <c r="U14" s="25"/>
       <c r="V14" s="25"/>
@@ -20859,7 +20877,9 @@
       <c r="R15" s="25">
         <v>0</v>
       </c>
-      <c r="S15" s="25"/>
+      <c r="S15" s="25">
+        <v>0</v>
+      </c>
       <c r="T15" s="25"/>
       <c r="U15" s="25"/>
       <c r="V15" s="25"/>
@@ -21044,7 +21064,7 @@
       </c>
       <c r="S19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T19" s="26">
         <f t="shared" si="1"/>

</xml_diff>